<commit_message>
executable file for distribution
</commit_message>
<xml_diff>
--- a/Excel-Documents/Sort_Time.xlsx
+++ b/Excel-Documents/Sort_Time.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ztben\workspace\FedExTrips\Excel-Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB8B94F0-80E1-44BB-B169-08AA8F19F69F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE00411-F3B9-46F5-A68D-E440F471E0B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3040" yWindow="3040" windowWidth="21600" windowHeight="12670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4180" yWindow="4180" windowWidth="21600" windowHeight="12670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="12" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="47">
   <si>
     <t>Flight 1460</t>
   </si>
@@ -166,13 +166,16 @@
     <t xml:space="preserve">Yes-explanation: </t>
   </si>
   <si>
-    <t>Total payload = 69,050</t>
-  </si>
-  <si>
-    <t>Heavyweight = 12,318</t>
-  </si>
-  <si>
-    <t>Express = 56,732</t>
+    <t xml:space="preserve">Actual = </t>
+  </si>
+  <si>
+    <t>Total payload = 53,946</t>
+  </si>
+  <si>
+    <t>Heavyweight = 13,240</t>
+  </si>
+  <si>
+    <t>Express = 40,706</t>
   </si>
 </sst>
 </file>
@@ -929,7 +932,7 @@
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -945,7 +948,7 @@
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -1137,17 +1140,17 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>